<commit_message>
local update before pull
</commit_message>
<xml_diff>
--- a/snapshot_report.xlsx
+++ b/snapshot_report.xlsx
@@ -806,10 +806,10 @@
         <v>2</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>10</v>
+        <v>10.5</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
@@ -887,7 +887,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>10.5</v>
+        <v>11</v>
       </c>
       <c r="C6" s="2" t="n">
         <v>24</v>
@@ -901,10 +901,10 @@
         <v>1</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>15</v>
+        <v>15.5</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
@@ -968,7 +968,7 @@
         <v>4</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>11</v>
+        <v>11.5</v>
       </c>
       <c r="C7" s="2" t="n">
         <v>24</v>
@@ -982,10 +982,10 @@
         <v>1.5</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
@@ -996,10 +996,10 @@
         <v>1</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>18</v>
+        <v>18.5</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
@@ -1049,7 +1049,7 @@
         <v>5</v>
       </c>
       <c r="B8" s="2" t="n">
-        <v>11.5</v>
+        <v>12</v>
       </c>
       <c r="C8" s="2" t="n">
         <v>24</v>
@@ -1063,7 +1063,7 @@
         <v>2</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>15.5</v>
+        <v>16.5</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>25</v>
@@ -1077,10 +1077,10 @@
         <v>1.5</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
@@ -1094,7 +1094,7 @@
         <v>12</v>
       </c>
       <c r="O8" s="2" t="n">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
@@ -1108,7 +1108,7 @@
         <v>14</v>
       </c>
       <c r="S8" s="2" t="n">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="T8" s="2" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
         <v>2</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>25</v>
@@ -1162,10 +1162,10 @@
         <v>2</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>18</v>
+        <v>19.5</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
@@ -1179,7 +1179,7 @@
         <v>12</v>
       </c>
       <c r="O9" s="2" t="n">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="P9" s="2" t="inlineStr">
         <is>
@@ -1190,10 +1190,10 @@
         <v>0</v>
       </c>
       <c r="R9" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="S9" s="2" t="n">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="T9" s="2" t="inlineStr">
         <is>
@@ -1230,10 +1230,10 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>2.98</v>
+        <v>3</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>16.5</v>
+        <v>17</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>25</v>
@@ -1247,10 +1247,10 @@
         <v>2</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>18</v>
+        <v>19.5</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
@@ -1261,10 +1261,10 @@
         <v>1.5</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>12</v>
+        <v>12.5</v>
       </c>
       <c r="O10" s="2" t="n">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="P10" s="2" t="inlineStr">
         <is>
@@ -1275,10 +1275,10 @@
         <v>0.5</v>
       </c>
       <c r="R10" s="2" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="S10" s="2" t="n">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="T10" s="2" t="inlineStr">
         <is>
@@ -1290,12 +1290,12 @@
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>R1/59 R4/60 R5/120</t>
+          <t>R1/60 R4/60 R5/120</t>
         </is>
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>R2/60 R3/59</t>
+          <t>R2/60 R3/60</t>
         </is>
       </c>
     </row>
@@ -1315,7 +1315,7 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>3.98</v>
+        <v>4</v>
       </c>
       <c r="F11" s="2" t="n">
         <v>17</v>
@@ -1332,10 +1332,10 @@
         <v>2</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>18</v>
+        <v>19.5</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
@@ -1346,10 +1346,10 @@
         <v>1.5</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="O11" s="2" t="n">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="P11" s="2" t="inlineStr">
         <is>
@@ -1360,10 +1360,10 @@
         <v>1</v>
       </c>
       <c r="R11" s="2" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="S11" s="2" t="n">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="T11" s="2" t="inlineStr">
         <is>
@@ -1375,12 +1375,12 @@
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>R1/119 R4/120 R5/180</t>
+          <t>R1/120 R4/0 R5/180</t>
         </is>
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>R2/120 R3/119</t>
+          <t>R2/120 R3/120</t>
         </is>
       </c>
     </row>
@@ -1400,7 +1400,7 @@
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>4.98</v>
+        <v>5</v>
       </c>
       <c r="F12" s="2" t="n">
         <v>17.5</v>
@@ -1417,38 +1417,38 @@
         <v>2.5</v>
       </c>
       <c r="J12" s="2" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="K12" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>MID</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="O12" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>MID</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R12" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="K12" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="n">
-        <v>1.98</v>
-      </c>
-      <c r="N12" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="O12" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="P12" s="2" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
-      <c r="Q12" s="2" t="n">
-        <v>1.02</v>
-      </c>
-      <c r="R12" s="2" t="n">
-        <v>14</v>
-      </c>
       <c r="S12" s="2" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="T12" s="2" t="inlineStr">
         <is>
@@ -1456,16 +1456,16 @@
         </is>
       </c>
       <c r="U12" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>R1/179 R2/60 R3/58</t>
+          <t>R1/180 R2/60 R5/240</t>
         </is>
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>R4/58 R5/60</t>
+          <t>R3/180 R4/60</t>
         </is>
       </c>
     </row>
@@ -1485,7 +1485,7 @@
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>5.98</v>
+        <v>6</v>
       </c>
       <c r="F13" s="2" t="n">
         <v>18</v>
@@ -1502,10 +1502,10 @@
         <v>3</v>
       </c>
       <c r="J13" s="2" t="n">
-        <v>18</v>
+        <v>19.5</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
@@ -1513,13 +1513,13 @@
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>2.48</v>
+        <v>1.5</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="O13" s="2" t="n">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="P13" s="2" t="inlineStr">
         <is>
@@ -1527,13 +1527,13 @@
         </is>
       </c>
       <c r="Q13" s="2" t="n">
-        <v>1.02</v>
+        <v>1</v>
       </c>
       <c r="R13" s="2" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="S13" s="2" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="T13" s="2" t="inlineStr">
         <is>
@@ -1541,16 +1541,16 @@
         </is>
       </c>
       <c r="U13" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="V13" t="inlineStr">
         <is>
-          <t>R1/239 R2/120 R3/118</t>
+          <t>R1/240 R2/120 R5/300</t>
         </is>
       </c>
       <c r="W13" t="inlineStr">
         <is>
-          <t>R4/118 R5/120</t>
+          <t>R3/240 R4/120</t>
         </is>
       </c>
     </row>
@@ -1570,10 +1570,10 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>5.98</v>
+        <v>7</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>18.5</v>
+        <v>18</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>25</v>
@@ -1584,13 +1584,13 @@
         </is>
       </c>
       <c r="I14" s="2" t="n">
-        <v>3.51</v>
+        <v>3</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>18</v>
+        <v>19.5</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
@@ -1598,10 +1598,10 @@
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>2.99</v>
+        <v>1.5</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="O14" s="2" t="n">
         <v>21</v>
@@ -1612,13 +1612,13 @@
         </is>
       </c>
       <c r="Q14" s="2" t="n">
-        <v>1.02</v>
+        <v>2</v>
       </c>
       <c r="R14" s="2" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="S14" s="2" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="T14" s="2" t="inlineStr">
         <is>
@@ -1626,16 +1626,16 @@
         </is>
       </c>
       <c r="U14" s="2" t="n">
-        <v>4.02</v>
+        <v>6</v>
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>R2/60 R3/60 R5/60</t>
+          <t>R1/300 R4/60 R5/360</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>R1/61 R4/60</t>
+          <t>R2/60 R3/60</t>
         </is>
       </c>
     </row>
@@ -1655,10 +1655,10 @@
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>25</v>
@@ -1669,13 +1669,13 @@
         </is>
       </c>
       <c r="I15" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>18</v>
+        <v>19.5</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
@@ -1683,10 +1683,10 @@
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>3.49</v>
+        <v>1.5</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="O15" s="2" t="n">
         <v>21</v>
@@ -1697,13 +1697,13 @@
         </is>
       </c>
       <c r="Q15" s="2" t="n">
-        <v>1.02</v>
+        <v>3</v>
       </c>
       <c r="R15" s="2" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="S15" s="2" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="T15" s="2" t="inlineStr">
         <is>
@@ -1711,16 +1711,16 @@
         </is>
       </c>
       <c r="U15" s="2" t="n">
-        <v>5.02</v>
+        <v>7</v>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>R1/1 R3/120 R5/120</t>
+          <t>R1/360 R4/120 R5/420</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>R2/1 R4/120</t>
+          <t>R2/120 R3/120</t>
         </is>
       </c>
     </row>
@@ -1740,27 +1740,27 @@
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F16" s="2" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>MID</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J16" s="2" t="n">
         <v>19.5</v>
       </c>
-      <c r="G16" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="n">
-        <v>4.49</v>
-      </c>
-      <c r="J16" s="2" t="n">
-        <v>18</v>
-      </c>
       <c r="K16" s="2" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
@@ -1768,10 +1768,10 @@
         </is>
       </c>
       <c r="M16" s="2" t="n">
-        <v>3.49</v>
+        <v>1.5</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="O16" s="2" t="n">
         <v>21</v>
@@ -1782,13 +1782,13 @@
         </is>
       </c>
       <c r="Q16" s="2" t="n">
-        <v>2.02</v>
+        <v>4</v>
       </c>
       <c r="R16" s="2" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="S16" s="2" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="T16" s="2" t="inlineStr">
         <is>
@@ -1796,16 +1796,16 @@
         </is>
       </c>
       <c r="U16" s="2" t="n">
-        <v>5.02</v>
+        <v>7</v>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>R1/61 R2/60 R4/60</t>
+          <t>R1/420 R2/60 R4/180</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>R3/60 R5/59</t>
+          <t>R3/180 R5/60</t>
         </is>
       </c>
     </row>
@@ -1825,10 +1825,10 @@
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>8.02</v>
+        <v>10</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>20.5</v>
+        <v>19.5</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>25</v>
@@ -1839,13 +1839,13 @@
         </is>
       </c>
       <c r="I17" s="2" t="n">
-        <v>5.49</v>
+        <v>4.5</v>
       </c>
       <c r="J17" s="2" t="n">
-        <v>18</v>
+        <v>19.5</v>
       </c>
       <c r="K17" s="2" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
@@ -1853,10 +1853,10 @@
         </is>
       </c>
       <c r="M17" s="2" t="n">
-        <v>3.49</v>
+        <v>1.5</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O17" s="2" t="n">
         <v>21</v>
@@ -1867,13 +1867,13 @@
         </is>
       </c>
       <c r="Q17" s="2" t="n">
-        <v>3.03</v>
+        <v>5</v>
       </c>
       <c r="R17" s="2" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="S17" s="2" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="T17" s="2" t="inlineStr">
         <is>
@@ -1881,16 +1881,16 @@
         </is>
       </c>
       <c r="U17" s="2" t="n">
-        <v>5.02</v>
+        <v>7</v>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>R2/60 R4/121 R5/0</t>
+          <t>R1/480 R2/60 R4/240</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>R1/0 R3/60</t>
+          <t>R3/60 R5/120</t>
         </is>
       </c>
     </row>
@@ -1910,10 +1910,10 @@
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>8.02</v>
+        <v>11</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>21.5</v>
+        <v>20.5</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>25</v>
@@ -1924,24 +1924,24 @@
         </is>
       </c>
       <c r="I18" s="2" t="n">
-        <v>6.49</v>
+        <v>5.5</v>
       </c>
       <c r="J18" s="2" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="K18" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>MID</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="N18" s="2" t="n">
         <v>18</v>
-      </c>
-      <c r="K18" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="L18" s="2" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="n">
-        <v>3.49</v>
-      </c>
-      <c r="N18" s="2" t="n">
-        <v>17</v>
       </c>
       <c r="O18" s="2" t="n">
         <v>21</v>
@@ -1952,13 +1952,13 @@
         </is>
       </c>
       <c r="Q18" s="2" t="n">
-        <v>4.03</v>
+        <v>6</v>
       </c>
       <c r="R18" s="2" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="S18" s="2" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="T18" s="2" t="inlineStr">
         <is>
@@ -1966,16 +1966,16 @@
         </is>
       </c>
       <c r="U18" s="2" t="n">
-        <v>5.52</v>
+        <v>7</v>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>R2/120 R4/181 R5/60</t>
+          <t>R1/540 R2/120 R4/300</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>R1/60 R3/120</t>
+          <t>R3/120 R5/180</t>
         </is>
       </c>
     </row>
@@ -1984,7 +1984,7 @@
         <v>16</v>
       </c>
       <c r="B19" s="2" t="n">
-        <v>22</v>
+        <v>20.5</v>
       </c>
       <c r="C19" s="2" t="n">
         <v>22</v>
@@ -1995,10 +1995,10 @@
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>8.02</v>
+        <v>11</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>22.5</v>
+        <v>21.5</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>25</v>
@@ -2009,13 +2009,13 @@
         </is>
       </c>
       <c r="I19" s="2" t="n">
-        <v>7.49</v>
+        <v>6.5</v>
       </c>
       <c r="J19" s="2" t="n">
-        <v>18</v>
+        <v>19.5</v>
       </c>
       <c r="K19" s="2" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
@@ -2023,10 +2023,10 @@
         </is>
       </c>
       <c r="M19" s="2" t="n">
-        <v>3.49</v>
+        <v>1.5</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O19" s="2" t="n">
         <v>21</v>
@@ -2037,13 +2037,13 @@
         </is>
       </c>
       <c r="Q19" s="2" t="n">
-        <v>5.03</v>
+        <v>7</v>
       </c>
       <c r="R19" s="2" t="n">
-        <v>14</v>
+        <v>21.5</v>
       </c>
       <c r="S19" s="2" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="T19" s="2" t="inlineStr">
         <is>
@@ -2051,11 +2051,11 @@
         </is>
       </c>
       <c r="U19" s="2" t="n">
-        <v>6.02</v>
+        <v>7.5</v>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>R2/180 R4/241 R5/120</t>
+          <t>R2/180 R4/360 R5/60</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
@@ -2069,7 +2069,7 @@
         <v>17</v>
       </c>
       <c r="B20" s="2" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C20" s="2" t="n">
         <v>22</v>
@@ -2080,10 +2080,10 @@
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>8.02</v>
+        <v>11</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>23.5</v>
+        <v>22.5</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>25</v>
@@ -2094,13 +2094,13 @@
         </is>
       </c>
       <c r="I20" s="2" t="n">
-        <v>8.49</v>
+        <v>7.5</v>
       </c>
       <c r="J20" s="2" t="n">
-        <v>18</v>
+        <v>19.5</v>
       </c>
       <c r="K20" s="2" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
@@ -2108,10 +2108,10 @@
         </is>
       </c>
       <c r="M20" s="2" t="n">
-        <v>3.49</v>
+        <v>1.5</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="O20" s="2" t="n">
         <v>21</v>
@@ -2122,13 +2122,13 @@
         </is>
       </c>
       <c r="Q20" s="2" t="n">
-        <v>6.03</v>
+        <v>8</v>
       </c>
       <c r="R20" s="2" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="S20" s="2" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="T20" s="2" t="inlineStr">
         <is>
@@ -2136,11 +2136,11 @@
         </is>
       </c>
       <c r="U20" s="2" t="n">
-        <v>6.52</v>
+        <v>8</v>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>R2/240 R4/301 R5/180</t>
+          <t>R2/240 R4/420 R5/120</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
@@ -2154,7 +2154,7 @@
         <v>18</v>
       </c>
       <c r="B21" s="2" t="n">
-        <v>22</v>
+        <v>19.5</v>
       </c>
       <c r="C21" s="2" t="n">
         <v>22</v>
@@ -2165,10 +2165,10 @@
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>8.02</v>
+        <v>11</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>24.5</v>
+        <v>23.5</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>25</v>
@@ -2179,13 +2179,13 @@
         </is>
       </c>
       <c r="I21" s="2" t="n">
-        <v>9.49</v>
+        <v>8.5</v>
       </c>
       <c r="J21" s="2" t="n">
-        <v>18</v>
+        <v>19.5</v>
       </c>
       <c r="K21" s="2" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
@@ -2193,10 +2193,10 @@
         </is>
       </c>
       <c r="M21" s="2" t="n">
-        <v>3.49</v>
+        <v>1.5</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="O21" s="2" t="n">
         <v>21</v>
@@ -2207,13 +2207,13 @@
         </is>
       </c>
       <c r="Q21" s="2" t="n">
-        <v>7.03</v>
+        <v>9</v>
       </c>
       <c r="R21" s="2" t="n">
-        <v>14</v>
+        <v>21.5</v>
       </c>
       <c r="S21" s="2" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="T21" s="2" t="inlineStr">
         <is>
@@ -2221,11 +2221,11 @@
         </is>
       </c>
       <c r="U21" s="2" t="n">
-        <v>6.52</v>
+        <v>8</v>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>R2/300 R4/361</t>
+          <t>R2/300 R4/480</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
@@ -2239,7 +2239,7 @@
         <v>19</v>
       </c>
       <c r="B22" s="2" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C22" s="2" t="n">
         <v>22</v>
@@ -2250,10 +2250,10 @@
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>8.02</v>
+        <v>11</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>25</v>
+        <v>24.5</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>25</v>
@@ -2264,13 +2264,13 @@
         </is>
       </c>
       <c r="I22" s="2" t="n">
-        <v>9.970000000000001</v>
+        <v>9.5</v>
       </c>
       <c r="J22" s="2" t="n">
-        <v>18</v>
+        <v>20.5</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
@@ -2278,10 +2278,10 @@
         </is>
       </c>
       <c r="M22" s="2" t="n">
-        <v>4.49</v>
+        <v>2.5</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>21</v>
+        <v>20.5</v>
       </c>
       <c r="O22" s="2" t="n">
         <v>21</v>
@@ -2292,13 +2292,13 @@
         </is>
       </c>
       <c r="Q22" s="2" t="n">
-        <v>8.029999999999999</v>
+        <v>9</v>
       </c>
       <c r="R22" s="2" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="S22" s="2" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="T22" s="2" t="inlineStr">
         <is>
@@ -2306,11 +2306,11 @@
         </is>
       </c>
       <c r="U22" s="2" t="n">
-        <v>6.52</v>
+        <v>8</v>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>R3/60 R4/421</t>
+          <t>R2/360 R3/60</t>
         </is>
       </c>
       <c r="W22" t="inlineStr"/>
@@ -2320,21 +2320,21 @@
         <v>20</v>
       </c>
       <c r="B23" s="2" t="n">
-        <v>22</v>
+        <v>19.5</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>MID</t>
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>9.02</v>
+        <v>11.5</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>25</v>
+        <v>24.8</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>25</v>
@@ -2345,13 +2345,13 @@
         </is>
       </c>
       <c r="I23" s="2" t="n">
-        <v>9.970000000000001</v>
+        <v>10</v>
       </c>
       <c r="J23" s="2" t="n">
-        <v>18</v>
+        <v>21.5</v>
       </c>
       <c r="K23" s="2" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
@@ -2359,10 +2359,10 @@
         </is>
       </c>
       <c r="M23" s="2" t="n">
-        <v>5.49</v>
+        <v>3.5</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>21.5</v>
+        <v>20.8</v>
       </c>
       <c r="O23" s="2" t="n">
         <v>25</v>
@@ -2373,13 +2373,13 @@
         </is>
       </c>
       <c r="Q23" s="2" t="n">
-        <v>8.52</v>
+        <v>9.25</v>
       </c>
       <c r="R23" s="2" t="n">
-        <v>14</v>
+        <v>20.5</v>
       </c>
       <c r="S23" s="2" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="T23" s="2" t="inlineStr">
         <is>
@@ -2387,11 +2387,11 @@
         </is>
       </c>
       <c r="U23" s="2" t="n">
-        <v>6.52</v>
+        <v>8</v>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>R1/60 R3/120 R4/59</t>
+          <t>R1/60 R3/120 R4/510</t>
         </is>
       </c>
       <c r="W23" t="inlineStr"/>
@@ -2401,21 +2401,21 @@
         <v>21</v>
       </c>
       <c r="B24" s="2" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>MID</t>
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>10.02</v>
+        <v>12</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>25</v>
+        <v>24.3</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>25</v>
@@ -2426,13 +2426,13 @@
         </is>
       </c>
       <c r="I24" s="2" t="n">
-        <v>9.970000000000001</v>
+        <v>10</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>18</v>
+        <v>22.5</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
@@ -2440,10 +2440,10 @@
         </is>
       </c>
       <c r="M24" s="2" t="n">
-        <v>6.49</v>
+        <v>4.5</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>22</v>
+        <v>21.2</v>
       </c>
       <c r="O24" s="2" t="n">
         <v>25</v>
@@ -2454,13 +2454,13 @@
         </is>
       </c>
       <c r="Q24" s="2" t="n">
-        <v>9.02</v>
+        <v>9.75</v>
       </c>
       <c r="R24" s="2" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="T24" s="2" t="inlineStr">
         <is>
@@ -2468,11 +2468,11 @@
         </is>
       </c>
       <c r="U24" s="2" t="n">
-        <v>6.52</v>
+        <v>8</v>
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>R1/120 R3/180 R4/119</t>
+          <t>R1/120 R3/180 R4/570</t>
         </is>
       </c>
       <c r="W24" t="inlineStr"/>
@@ -2482,21 +2482,21 @@
         <v>22</v>
       </c>
       <c r="B25" s="2" t="n">
-        <v>22</v>
+        <v>20.5</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>MID</t>
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>11.02</v>
+        <v>12.5</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>25</v>
+        <v>24.5</v>
       </c>
       <c r="G25" s="2" t="n">
         <v>25</v>
@@ -2507,13 +2507,13 @@
         </is>
       </c>
       <c r="I25" s="2" t="n">
-        <v>9.970000000000001</v>
+        <v>10.25</v>
       </c>
       <c r="J25" s="2" t="n">
-        <v>18</v>
+        <v>22.8</v>
       </c>
       <c r="K25" s="2" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
@@ -2521,10 +2521,10 @@
         </is>
       </c>
       <c r="M25" s="2" t="n">
-        <v>7.49</v>
+        <v>5</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>22.5</v>
+        <v>21.7</v>
       </c>
       <c r="O25" s="2" t="n">
         <v>25</v>
@@ -2535,13 +2535,13 @@
         </is>
       </c>
       <c r="Q25" s="2" t="n">
-        <v>9.52</v>
+        <v>10.25</v>
       </c>
       <c r="R25" s="2" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="S25" s="2" t="n">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="T25" s="2" t="inlineStr">
         <is>
@@ -2549,16 +2549,16 @@
         </is>
       </c>
       <c r="U25" s="2" t="n">
-        <v>6.52</v>
+        <v>8</v>
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>R1/180 R3/240 R4/179</t>
+          <t>R1/180 R2/420 R4/630</t>
         </is>
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>R2/60 R5/60</t>
+          <t>R5/60</t>
         </is>
       </c>
     </row>
@@ -2567,18 +2567,18 @@
         <v>23</v>
       </c>
       <c r="B26" s="2" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>MID</t>
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>12.02</v>
+        <v>13</v>
       </c>
       <c r="F26" s="2" t="n">
         <v>25</v>
@@ -2592,13 +2592,13 @@
         </is>
       </c>
       <c r="I26" s="2" t="n">
-        <v>9.970000000000001</v>
+        <v>10.75</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>18</v>
+        <v>22.3</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
@@ -2606,10 +2606,10 @@
         </is>
       </c>
       <c r="M26" s="2" t="n">
-        <v>8.49</v>
+        <v>5</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>23</v>
+        <v>22.2</v>
       </c>
       <c r="O26" s="2" t="n">
         <v>25</v>
@@ -2620,13 +2620,13 @@
         </is>
       </c>
       <c r="Q26" s="2" t="n">
-        <v>10.02</v>
+        <v>10.75</v>
       </c>
       <c r="R26" s="2" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="S26" s="2" t="n">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="T26" s="2" t="inlineStr">
         <is>
@@ -2634,16 +2634,16 @@
         </is>
       </c>
       <c r="U26" s="2" t="n">
-        <v>6.52</v>
+        <v>8</v>
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>R1/240 R3/300 R4/239</t>
+          <t>R1/240 R2/390 R4/480</t>
         </is>
       </c>
       <c r="W26" t="inlineStr">
         <is>
-          <t>R2/120 R5/120</t>
+          <t>R5/0</t>
         </is>
       </c>
     </row>
@@ -2652,21 +2652,21 @@
         <v>24</v>
       </c>
       <c r="B27" s="2" t="n">
-        <v>22</v>
+        <v>21.3</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>MID</t>
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>12.02</v>
+        <v>13.26</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>25</v>
+        <v>24.5</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>25</v>
@@ -2677,13 +2677,13 @@
         </is>
       </c>
       <c r="I27" s="2" t="n">
-        <v>10.47</v>
+        <v>10.75</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>18</v>
+        <v>22.5</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
@@ -2691,10 +2691,10 @@
         </is>
       </c>
       <c r="M27" s="2" t="n">
-        <v>8.49</v>
+        <v>5.48</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>23.5</v>
+        <v>22.7</v>
       </c>
       <c r="O27" s="2" t="n">
         <v>25</v>
@@ -2705,13 +2705,13 @@
         </is>
       </c>
       <c r="Q27" s="2" t="n">
-        <v>10.52</v>
+        <v>11.25</v>
       </c>
       <c r="R27" s="2" t="n">
-        <v>14</v>
+        <v>20.5</v>
       </c>
       <c r="S27" s="2" t="n">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="T27" s="2" t="inlineStr">
         <is>
@@ -2719,16 +2719,16 @@
         </is>
       </c>
       <c r="U27" s="2" t="n">
-        <v>7.02</v>
+        <v>8.5</v>
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>R2/60 R4/299 R5/60</t>
+          <t>R3/239 R4/60 R5/60</t>
         </is>
       </c>
       <c r="W27" t="inlineStr">
         <is>
-          <t>R1/60 R3/60</t>
+          <t>R1/29</t>
         </is>
       </c>
     </row>
@@ -2737,21 +2737,21 @@
         <v>25</v>
       </c>
       <c r="B28" s="2" t="n">
-        <v>22</v>
+        <v>21.5</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>MID</t>
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>12.02</v>
+        <v>13.49</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>25</v>
@@ -2762,13 +2762,13 @@
         </is>
       </c>
       <c r="I28" s="2" t="n">
-        <v>10.97</v>
+        <v>10.75</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>18</v>
+        <v>22.8</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
@@ -2776,10 +2776,10 @@
         </is>
       </c>
       <c r="M28" s="2" t="n">
-        <v>8.49</v>
+        <v>6.02</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>24</v>
+        <v>23.2</v>
       </c>
       <c r="O28" s="2" t="n">
         <v>25</v>
@@ -2790,13 +2790,13 @@
         </is>
       </c>
       <c r="Q28" s="2" t="n">
-        <v>11.02</v>
+        <v>11.75</v>
       </c>
       <c r="R28" s="2" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="S28" s="2" t="n">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="T28" s="2" t="inlineStr">
         <is>
@@ -2804,39 +2804,35 @@
         </is>
       </c>
       <c r="U28" s="2" t="n">
-        <v>7.52</v>
+        <v>9</v>
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>R2/120 R4/359 R5/120</t>
-        </is>
-      </c>
-      <c r="W28" t="inlineStr">
-        <is>
-          <t>R1/120 R3/120</t>
-        </is>
-      </c>
+          <t>R1/28 R4/120 R5/120</t>
+        </is>
+      </c>
+      <c r="W28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
         <v>26</v>
       </c>
       <c r="B29" s="2" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>MID</t>
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>12.03</v>
+        <v>13.49</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>25</v>
+        <v>24.5</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>25</v>
@@ -2847,13 +2843,13 @@
         </is>
       </c>
       <c r="I29" s="2" t="n">
-        <v>10.97</v>
+        <v>11.24</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>18</v>
+        <v>22.3</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
@@ -2861,10 +2857,10 @@
         </is>
       </c>
       <c r="M29" s="2" t="n">
-        <v>8.51</v>
+        <v>6.02</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>24.5</v>
+        <v>23.7</v>
       </c>
       <c r="O29" s="2" t="n">
         <v>25</v>
@@ -2875,13 +2871,13 @@
         </is>
       </c>
       <c r="Q29" s="2" t="n">
-        <v>11.02</v>
+        <v>12.25</v>
       </c>
       <c r="R29" s="2" t="n">
-        <v>14</v>
+        <v>20.5</v>
       </c>
       <c r="S29" s="2" t="n">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="T29" s="2" t="inlineStr">
         <is>
@@ -2889,14 +2885,14 @@
         </is>
       </c>
       <c r="U29" s="2" t="n">
-        <v>7.52</v>
-      </c>
-      <c r="V29" t="inlineStr"/>
-      <c r="W29" t="inlineStr">
-        <is>
-          <t>R2/61 R4/61</t>
-        </is>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>R2/539 R4/180</t>
+        </is>
+      </c>
+      <c r="W29" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>